<commit_message>
Add member check page with Section-Element mapping and /post/TABLE support
- Add sidebar menu for member design check (부재검토)
- Add backend Section-Element mapping router (member.py)
- Add RC beam check page with section-based design result query
- Update EndpointForm to support /post/TABLE with auto-generated body
- Fix flattenResponse to handle HEAD+DATA response format

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/floor_load_template.xlsx
+++ b/backend/data/floor_load_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="현재_통합_문서" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bbf02a8dd7620d33/문서/PyQT Tutorial/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bbf02a8dd7620d33/문서/Task_MIDAS/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{020AFB63-AB9D-48A5-85FE-6CF65DAB25AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{020AFB63-AB9D-48A5-85FE-6CF65DAB25AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D90D082E-CB0B-406B-A702-731C9880A747}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{76AE1FC2-89F0-4A59-A031-040BA28C7032}"/>
   </bookViews>
@@ -37,6 +37,28 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -566,6 +588,69 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -583,69 +668,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="3" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -670,78 +692,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>182218</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>57977</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="262433" cy="271743"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4CD81AE5-11EF-4FC0-AFE8-8E821AF9F5D7}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="5059018" y="210377"/>
-          <a:ext cx="262433" cy="271743"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>397566</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>298175</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>173935</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1487330" cy="372474"/>
     <xdr:sp macro="" textlink="">
@@ -757,7 +710,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5274366" y="152400"/>
+          <a:off x="6932545" y="173935"/>
           <a:ext cx="1487330" cy="372474"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -825,14 +778,74 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -870,7 +883,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -976,7 +989,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1118,7 +1131,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1157,7 +1170,9 @@
       <c r="F2" s="9"/>
       <c r="G2" s="8"/>
       <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
+      <c r="I2" s="8" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="J2" s="8"/>
     </row>
     <row r="3" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1176,23 +1191,23 @@
       </c>
     </row>
     <row r="6" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="13"/>
-      <c r="D6" s="12" t="s">
+      <c r="C6" s="34"/>
+      <c r="D6" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="10" t="s">
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" s="31" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1215,525 +1230,539 @@
       <c r="G7" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="H7" s="15"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
     </row>
     <row r="8" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="12">
         <v>27</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="12">
         <v>5</v>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="13">
         <v>0.14000000000000001</v>
       </c>
-      <c r="H8" s="16" t="s">
+      <c r="H8" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="29"/>
     </row>
     <row r="9" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="24"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="26" t="s">
+      <c r="C9" s="27"/>
+      <c r="D9" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="27">
+      <c r="E9" s="15">
         <v>20</v>
       </c>
-      <c r="F9" s="27">
+      <c r="F9" s="15">
         <v>25</v>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="16">
         <v>0.5</v>
       </c>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
     </row>
     <row r="10" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="24"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="26" t="s">
+      <c r="C10" s="27"/>
+      <c r="D10" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="28">
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="16">
         <v>0.2</v>
       </c>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
     </row>
     <row r="11" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="24"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="31" t="s">
+      <c r="C11" s="27"/>
+      <c r="D11" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="32"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="33">
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="19">
         <v>0.84</v>
       </c>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="30"/>
     </row>
     <row r="12" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="24"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="26" t="s">
+      <c r="C12" s="27"/>
+      <c r="D12" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="27">
+      <c r="E12" s="15">
         <v>150</v>
       </c>
-      <c r="F12" s="27">
+      <c r="F12" s="15">
         <v>24</v>
       </c>
-      <c r="G12" s="28">
+      <c r="G12" s="16">
         <v>3.6</v>
       </c>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="30"/>
     </row>
     <row r="13" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="29"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="34" t="s">
+      <c r="B13" s="25"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="36">
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="22">
         <v>4.4400000000000004</v>
       </c>
-      <c r="H13" s="18">
+      <c r="H13" s="10">
         <v>4</v>
       </c>
-      <c r="I13" s="18">
+      <c r="I13" s="10">
         <v>8.44</v>
       </c>
-      <c r="J13" s="18">
+      <c r="J13" s="10">
         <v>11.73</v>
       </c>
     </row>
     <row r="14" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="12">
         <v>27</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="12">
         <v>5</v>
       </c>
-      <c r="G14" s="23">
+      <c r="G14" s="13">
         <v>0.14000000000000001</v>
       </c>
-      <c r="H14" s="16" t="s">
+      <c r="H14" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
     </row>
     <row r="15" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="24"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="26" t="s">
+      <c r="C15" s="27"/>
+      <c r="D15" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="E15" s="27">
+      <c r="E15" s="15">
         <v>20</v>
       </c>
-      <c r="F15" s="27">
+      <c r="F15" s="15">
         <v>25</v>
       </c>
-      <c r="G15" s="28">
+      <c r="G15" s="16">
         <v>0.5</v>
       </c>
-      <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
     </row>
     <row r="16" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="24"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="26" t="s">
+      <c r="C16" s="27"/>
+      <c r="D16" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="28">
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="16">
         <v>0.2</v>
       </c>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
     </row>
     <row r="17" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="24"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="31" t="s">
+      <c r="C17" s="27"/>
+      <c r="D17" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="33">
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="19">
         <v>0.84</v>
       </c>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="30"/>
     </row>
     <row r="18" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="24"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="26" t="s">
+      <c r="C18" s="27"/>
+      <c r="D18" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="15">
         <v>150</v>
       </c>
-      <c r="F18" s="27">
+      <c r="F18" s="15">
         <v>24</v>
       </c>
-      <c r="G18" s="28">
+      <c r="G18" s="16">
         <v>3.6</v>
       </c>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
     </row>
     <row r="19" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="29"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="34" t="s">
+      <c r="B19" s="25"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="36">
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="22">
         <v>4.4400000000000004</v>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="10">
         <v>3</v>
       </c>
-      <c r="I19" s="18">
+      <c r="I19" s="10">
         <v>7.44</v>
       </c>
-      <c r="J19" s="18">
+      <c r="J19" s="10">
         <v>10.130000000000001</v>
       </c>
     </row>
     <row r="20" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="22">
+      <c r="E20" s="12">
         <v>27</v>
       </c>
-      <c r="F20" s="22">
+      <c r="F20" s="12">
         <v>5</v>
       </c>
-      <c r="G20" s="23">
+      <c r="G20" s="13">
         <v>0.14000000000000001</v>
       </c>
-      <c r="H20" s="16" t="s">
+      <c r="H20" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
     </row>
     <row r="21" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="24"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="26" t="s">
+      <c r="C21" s="27"/>
+      <c r="D21" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="27">
+      <c r="E21" s="15">
         <v>20</v>
       </c>
-      <c r="F21" s="27">
+      <c r="F21" s="15">
         <v>25</v>
       </c>
-      <c r="G21" s="28">
+      <c r="G21" s="16">
         <v>0.5</v>
       </c>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="17"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="30"/>
+      <c r="J21" s="30"/>
     </row>
     <row r="22" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="24"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="26" t="s">
+      <c r="C22" s="27"/>
+      <c r="D22" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="28">
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="16">
         <v>0.2</v>
       </c>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="30"/>
+      <c r="J22" s="30"/>
     </row>
     <row r="23" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="29"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="34" t="s">
+      <c r="B23" s="25"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="36">
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="22">
         <v>0.84</v>
       </c>
-      <c r="H23" s="18">
+      <c r="H23" s="10">
         <v>3</v>
       </c>
-      <c r="I23" s="18">
+      <c r="I23" s="10">
         <v>3.84</v>
       </c>
-      <c r="J23" s="18">
+      <c r="J23" s="10">
         <v>5.81</v>
       </c>
     </row>
     <row r="24" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="21" t="s">
+      <c r="D24" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E24" s="22">
+      <c r="E24" s="12">
         <v>6</v>
       </c>
-      <c r="F24" s="22">
+      <c r="F24" s="12">
         <v>16</v>
       </c>
-      <c r="G24" s="23">
+      <c r="G24" s="13">
         <v>0.1</v>
       </c>
-      <c r="H24" s="16" t="s">
+      <c r="H24" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="I24" s="16"/>
-      <c r="J24" s="16"/>
+      <c r="I24" s="29"/>
+      <c r="J24" s="29"/>
     </row>
     <row r="25" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="24"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="26" t="s">
+      <c r="C25" s="27"/>
+      <c r="D25" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="E25" s="27">
+      <c r="E25" s="15">
         <v>24</v>
       </c>
-      <c r="F25" s="27">
+      <c r="F25" s="15">
         <v>20</v>
       </c>
-      <c r="G25" s="28">
+      <c r="G25" s="16">
         <v>0.48</v>
       </c>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="30"/>
+      <c r="J25" s="30"/>
     </row>
     <row r="26" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="24"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="26" t="s">
+      <c r="C26" s="27"/>
+      <c r="D26" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="E26" s="27">
+      <c r="E26" s="15">
         <v>10</v>
       </c>
-      <c r="F26" s="27">
+      <c r="F26" s="15">
         <v>20</v>
       </c>
-      <c r="G26" s="28">
+      <c r="G26" s="16">
         <v>0.2</v>
       </c>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="30"/>
+      <c r="J26" s="30"/>
     </row>
     <row r="27" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="24"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="26" t="s">
+      <c r="C27" s="27"/>
+      <c r="D27" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="28">
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="16">
         <v>0.2</v>
       </c>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="30"/>
+      <c r="J27" s="30"/>
     </row>
     <row r="28" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="24"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="31" t="s">
+      <c r="C28" s="27"/>
+      <c r="D28" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="33">
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="19">
         <v>0.98</v>
       </c>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="30"/>
     </row>
     <row r="29" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="24"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="26" t="s">
+      <c r="C29" s="27"/>
+      <c r="D29" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="E29" s="27">
+      <c r="E29" s="15">
         <v>150</v>
       </c>
-      <c r="F29" s="27">
+      <c r="F29" s="15">
         <v>24</v>
       </c>
-      <c r="G29" s="28">
+      <c r="G29" s="16">
         <v>3.6</v>
       </c>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
     </row>
     <row r="30" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="29"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="34" t="s">
+      <c r="B30" s="25"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="E30" s="35"/>
-      <c r="F30" s="35"/>
-      <c r="G30" s="36">
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="22">
         <v>4.58</v>
       </c>
-      <c r="H30" s="18">
+      <c r="H30" s="10">
         <v>1</v>
       </c>
-      <c r="I30" s="18">
+      <c r="I30" s="10">
         <v>5.58</v>
       </c>
-      <c r="J30" s="18">
+      <c r="J30" s="10">
         <v>7.1</v>
       </c>
     </row>
     <row r="31" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="20" t="s">
+      <c r="C31" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="D31" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
-      <c r="G31" s="23">
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="13">
         <v>0.1</v>
       </c>
-      <c r="H31" s="16" t="s">
+      <c r="H31" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="I31" s="16"/>
-      <c r="J31" s="16"/>
+      <c r="I31" s="29"/>
+      <c r="J31" s="29"/>
     </row>
     <row r="32" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="24"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="26" t="s">
+      <c r="C32" s="27"/>
+      <c r="D32" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="28">
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="16">
         <v>0.2</v>
       </c>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="17"/>
+      <c r="H32" s="30"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="30"/>
     </row>
     <row r="33" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="24"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="26" t="s">
+      <c r="C33" s="27"/>
+      <c r="D33" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="28">
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="16">
         <v>0.2</v>
       </c>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="30"/>
+      <c r="J33" s="30"/>
     </row>
     <row r="34" spans="2:10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="29"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="34" t="s">
+      <c r="B34" s="25"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
-      <c r="G34" s="36">
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="22">
         <v>0.5</v>
       </c>
-      <c r="H34" s="18">
+      <c r="H34" s="10">
         <v>1</v>
       </c>
-      <c r="I34" s="18">
+      <c r="I34" s="10">
         <v>1.5</v>
       </c>
-      <c r="J34" s="18">
+      <c r="J34" s="10">
         <v>2.2000000000000002</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="B8:B13"/>
+    <mergeCell ref="C8:C13"/>
+    <mergeCell ref="B24:B30"/>
+    <mergeCell ref="C24:C30"/>
+    <mergeCell ref="H14:H18"/>
+    <mergeCell ref="H8:H12"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="C14:C19"/>
+    <mergeCell ref="H20:H22"/>
     <mergeCell ref="B31:B34"/>
     <mergeCell ref="C31:C34"/>
     <mergeCell ref="J8:J12"/>
@@ -1750,20 +1779,6 @@
     <mergeCell ref="B20:B23"/>
     <mergeCell ref="C20:C23"/>
     <mergeCell ref="H24:H29"/>
-    <mergeCell ref="B24:B30"/>
-    <mergeCell ref="C24:C30"/>
-    <mergeCell ref="H14:H18"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:G6"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="B8:B13"/>
-    <mergeCell ref="C8:C13"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="C14:C19"/>
-    <mergeCell ref="H20:H22"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>